<commit_message>
Terreo: banheiro sai da parede da garagem; banheiro + lavabo no fundo da cozinha (faixa SO) c/ janelas p/ o acesso lateral e porta do lavabo p/ o quintal
</commit_message>
<xml_diff>
--- a/planilha-q22-l8.xlsx
+++ b/planilha-q22-l8.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resumo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Etapas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Itens" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cotações" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Comparativo" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Revisões" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Fornecedores" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Etapas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Itens" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cotações" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparativo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revisões" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fornecedores" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -614,7 +614,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Gerada em 16/07/2026 02:02 (BRT)</t>
+          <t>Gerada em 16/07/2026 13:49 (BRT)</t>
         </is>
       </c>
     </row>
@@ -927,6 +927,18 @@
       <c r="B26" s="12" t="inlineStr">
         <is>
           <t>Radier ~103 m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Térreo — faixa SO</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>Despensa + banheiro completo (1,50 × 2,20) + lavabo (1,50 × 1,50) no fundo da cozinha · janelas p/ o acesso lateral · porta do lavabo direto p/ a varanda gourmet</t>
         </is>
       </c>
     </row>
@@ -947,11 +959,12 @@
     <row r="31"/>
     <row r="32"/>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A30:D32"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B27:D27"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="B25:D25"/>
     <mergeCell ref="B24:D24"/>
@@ -1844,7 +1857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M146"/>
+  <dimension ref="A1:M149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4230,7 +4243,7 @@
       </c>
       <c r="M44" s="21" t="inlineStr">
         <is>
-          <t>suíte, banheiro do quarto e banheiro térreo · caimento 2% na impermeabilização</t>
+          <t>suíte, banheiro do quarto e banheiro do térreo (agora no fundo da cozinha, faixa SO)</t>
         </is>
       </c>
     </row>
@@ -10037,6 +10050,179 @@
       <c r="M146" s="21" t="inlineStr">
         <is>
           <t>cotar empreiteiro/equipe separadamente do material · preencher o Fornecedor</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="16" t="inlineStr">
+        <is>
+          <t>IT144</t>
+        </is>
+      </c>
+      <c r="B147" s="17" t="inlineStr">
+        <is>
+          <t>Hidráulica</t>
+        </is>
+      </c>
+      <c r="C147" s="17" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D147" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="E147" s="16" t="inlineStr">
+        <is>
+          <t>Lavabo do térreo — vaso + cuba + torneira + sifão</t>
+        </is>
+      </c>
+      <c r="F147" s="16" t="inlineStr">
+        <is>
+          <t>lavabo 1,50 × 1,50 no canto SO/SE, porta p/ a varanda</t>
+        </is>
+      </c>
+      <c r="G147" s="16" t="inlineStr">
+        <is>
+          <t>cj</t>
+        </is>
+      </c>
+      <c r="H147" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="I147" s="16">
+        <f>COUNTIFS(Cotações!$E$2:$E$2,$A147)</f>
+        <v/>
+      </c>
+      <c r="J147" s="32">
+        <f>IF(I147=0,"—",_xlfn.MINIFS(Cotações!$J$2:$J$2,Cotações!$E$2:$E$2,$A147))</f>
+        <v/>
+      </c>
+      <c r="K147" s="17">
+        <f>IF(I147=0,"—",IFERROR(INDEX(Cotações!$H$2:$H$2,MATCH(1,INDEX((Cotações!$E$2:$E$2=$A147)*(Cotações!$J$2:$J$2=J147),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="L147" s="18">
+        <f>IF(I147=0,"—",IFERROR(J147*H147,""))</f>
+        <v/>
+      </c>
+      <c r="M147" s="16" t="inlineStr">
+        <is>
+          <t>ponto novo: ramal de esgoto e água aproveita a prumada do banheiro vizinho (paredes coladas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="21" t="inlineStr">
+        <is>
+          <t>IT145</t>
+        </is>
+      </c>
+      <c r="B148" s="22" t="inlineStr">
+        <is>
+          <t>Hidráulica</t>
+        </is>
+      </c>
+      <c r="C148" s="22" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D148" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="E148" s="21" t="inlineStr">
+        <is>
+          <t>Ramal hidráulico do lavabo (água fria + esgoto + ventilação)</t>
+        </is>
+      </c>
+      <c r="F148" s="21" t="inlineStr"/>
+      <c r="G148" s="21" t="inlineStr">
+        <is>
+          <t>vb</t>
+        </is>
+      </c>
+      <c r="H148" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="I148" s="21">
+        <f>COUNTIFS(Cotações!$E$2:$E$2,$A148)</f>
+        <v/>
+      </c>
+      <c r="J148" s="30">
+        <f>IF(I148=0,"—",_xlfn.MINIFS(Cotações!$J$2:$J$2,Cotações!$E$2:$E$2,$A148))</f>
+        <v/>
+      </c>
+      <c r="K148" s="22">
+        <f>IF(I148=0,"—",IFERROR(INDEX(Cotações!$H$2:$H$2,MATCH(1,INDEX((Cotações!$E$2:$E$2=$A148)*(Cotações!$J$2:$J$2=J148),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="L148" s="23">
+        <f>IF(I148=0,"—",IFERROR(J148*H148,""))</f>
+        <v/>
+      </c>
+      <c r="M148" s="21" t="inlineStr">
+        <is>
+          <t>economia: banheiro e lavabo compartilham a mesma parede hidráulica</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="16" t="inlineStr">
+        <is>
+          <t>IT146</t>
+        </is>
+      </c>
+      <c r="B149" s="17" t="inlineStr">
+        <is>
+          <t>Geral / Estrutura</t>
+        </is>
+      </c>
+      <c r="C149" s="17" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="D149" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="E149" s="16" t="inlineStr">
+        <is>
+          <t>Acabamento do lavabo do térreo — microcimento + piso resinado</t>
+        </is>
+      </c>
+      <c r="F149" s="16" t="inlineStr">
+        <is>
+          <t>paredes + piso · sem carpete de pedra (lavabo seco)</t>
+        </is>
+      </c>
+      <c r="G149" s="16" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="H149" s="31" t="n">
+        <v>9</v>
+      </c>
+      <c r="I149" s="16">
+        <f>COUNTIFS(Cotações!$E$2:$E$2,$A149)</f>
+        <v/>
+      </c>
+      <c r="J149" s="32">
+        <f>IF(I149=0,"—",_xlfn.MINIFS(Cotações!$J$2:$J$2,Cotações!$E$2:$E$2,$A149))</f>
+        <v/>
+      </c>
+      <c r="K149" s="17">
+        <f>IF(I149=0,"—",IFERROR(INDEX(Cotações!$H$2:$H$2,MATCH(1,INDEX((Cotações!$E$2:$E$2=$A149)*(Cotações!$J$2:$J$2=J149),0),0)),""))</f>
+        <v/>
+      </c>
+      <c r="L149" s="18">
+        <f>IF(I149=0,"—",IFERROR(J149*H149,""))</f>
+        <v/>
+      </c>
+      <c r="M149" s="16" t="inlineStr">
+        <is>
+          <t>DIY viável — ambiente pequeno e sem área molhada</t>
         </is>
       </c>
     </row>
@@ -10615,7 +10801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10865,6 +11051,23 @@
       <c r="C15" s="17" t="inlineStr">
         <is>
           <t>Material e mão de obra separados por etapa e por fornecedor</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>16/07/2026</t>
+        </is>
+      </c>
+      <c r="B16" s="22" t="inlineStr">
+        <is>
+          <t>Térreo: banheiro sai da parede da garagem → banheiro + lavabo no fundo da cozinha (faixa SO)</t>
+        </is>
+      </c>
+      <c r="C16" s="22" t="inlineStr">
+        <is>
+          <t>Cozinha 36 → 29 m² · +1 lavabo · janelas p/ o acesso lateral · porta do lavabo p/ a varanda</t>
         </is>
       </c>
     </row>

</xml_diff>